<commit_message>
Removed Width and Depths
</commit_message>
<xml_diff>
--- a/residual_stress_maraging_steel_dataset.xlsx
+++ b/residual_stress_maraging_steel_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ragha\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Code\PYTHON\MS300-LPBF-Prorperties-Prediction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272793D7-86CD-4F6C-B9A2-6FFEE3DA0632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59369757-B7C2-42BB-AB7F-890AA9932195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{A0F8BB14-5D3E-4697-8EA2-375B6861484F}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>StdOrder</t>
   </si>
@@ -64,12 +64,15 @@
   <si>
     <t>ED</t>
   </si>
+  <si>
+    <t>Experimental</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,6 +85,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -131,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -140,6 +151,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1484,7 +1496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8049C93D-E3F8-4950-8F41-3A8F9EF24FC2}">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="9" max="9" width="12.6328125" bestFit="1" customWidth="1"/>
@@ -2432,6 +2444,25 @@
       </c>
       <c r="N21">
         <v>-907.97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="37" x14ac:dyDescent="0.85">
+      <c r="E27" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="E28">
+        <v>285</v>
+      </c>
+      <c r="F28">
+        <v>960</v>
+      </c>
+      <c r="G28">
+        <v>0.11</v>
+      </c>
+      <c r="I28">
+        <v>-405</v>
       </c>
     </row>
   </sheetData>
@@ -3216,23 +3247,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010009195B83481AFA4CAA5912DB215B0890" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="86c78988e6ae14f99ea4a576a843ebab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bbc0aaf6cedd4663464e8562c032f235" ns3:_="">
     <xsd:import namespace="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca"/>
@@ -3432,10 +3446,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C01F79D1-F162-4498-AA86-D8095413B880}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B8660BA-057A-4FEB-8387-5D42A86A4560}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3457,19 +3498,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B8660BA-057A-4FEB-8387-5D42A86A4560}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C01F79D1-F162-4498-AA86-D8095413B880}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2e69ede7-b5e3-47d1-8889-c5b647cbc3ca"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>